<commit_message>
fix: allow empty user lists without falling back to seed users, clear all user registrations
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -397,62 +397,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E3"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Username</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Password</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Role</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Room</v>
-      </c>
-      <c r="E1" t="str">
-        <v>CreatedAt</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>giao-vien-1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>123</v>
-      </c>
-      <c r="C2" t="str">
-        <v>teacher</v>
-      </c>
-      <c r="D2" t="str">
-        <v>64CTT1</v>
-      </c>
-      <c r="E2" t="str">
-        <v>2026-06-03T14:55:41.558Z</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>hoc-sinh-1</v>
-      </c>
-      <c r="B3" t="str">
-        <v>123</v>
-      </c>
-      <c r="C3" t="str">
-        <v>student</v>
-      </c>
-      <c r="D3" t="str">
-        <v>64CTT1</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-06-03T14:55:41.558Z</v>
-      </c>
-    </row>
-  </sheetData>
+  <dimension ref="A1"/>
+  <sheetData/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>